<commit_message>
Add Santa logistics-lever analysis
Last season logistics was 282 RUB/unit vs 82 RUB/unit margin (3.4x) due
to товар not spread across clusters -> long-distance delivery. Local FBO
distribution could cut logistics to ~150/unit, lifting margin to ~214/unit
= ~1.05M season margin on same volume (vs 402k), before volume uplift.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0153XBqtvJYtRAKHdw3RmMsz
</commit_message>
<xml_diff>
--- a/outputs/ozon_sales_plan/ozon_santa_q4_2026.xlsx
+++ b/outputs/ozon_sales_plan/ozon_santa_q4_2026.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Деды Морозы — прошлый сезон" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Логистика — рычаг" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -93,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -107,6 +108,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -774,4 +781,235 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Деды Морозы: логистика — главный рычаг прибыли</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Прошлый сезон товар не был разложен по кластерам → дальняя доставка → логистика 282 ₽/шт съела маржу.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Показатель (на 1 шт)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Прошлый сезон (факт)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Этот сезон (локально)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Разница</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Выручка</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>1437</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>1437</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Комиссия (40%)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>-577</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>-577</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Себестоимость</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>-294</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>-294</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Логистика</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>-282</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>-150</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Прочее (эквайринг и др.)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>-202</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>-202</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>МАРЖА / шт</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>214</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>На объёме прошлого сезона (4 905 шт):</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Маржа прошлый сезон (факт)</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>401404</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Маржа при локальной раскладке (та же продажа)</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>1049670</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Прирост только от логистики</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>648266</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>ВЫВОД: логистика (282 ₽/шт) была в 3,4 раза больше маржи (82 ₽/шт). Главное действие сезона — разложить Санту по кластерам спроса.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Приоритет складов (по спросу категории): Москва+МО, СПб, Ростов, Казань, Новосибирск, Екатеринбург, Краснодар — как в плане FBO по косметике.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Эффект двойной: (1) логистика/шт падает → маржа/шт растёт ~×2,6; (2) локальное наличие → короткая доставка → выше конверсия и объём.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Цель сезона: не 402 тыс., а ориентир ~1 млн+ маржи только за счёт логистики, плюс рост объёма сверху.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Параметр 150 ₽/шт — консервативная оценка локальной логистики; уточним по тарифам FBO Ozon для габаритных (КГТ).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A19:D19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>